<commit_message>
feat: update subscription model to include discount and adjust status handling
- Added discount field to Subscription interface and parsing logic.
- Updated test scenarios to reflect changes in subscription statuses, removing paused subscriptions.
- Modified utility functions to handle subscription status checks without paused state.
- Adjusted related tests and data to ensure consistency with new subscription logic.
</commit_message>
<xml_diff>
--- a/data/test/subscriptions.xlsx
+++ b/data/test/subscriptions.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M46"/>
+  <dimension ref="A1:M49"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -443,13 +443,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>e01d987d-6a5f-4f31-bd71-1486afa53c78</v>
+        <v>777f97b6-a669-4861-8b9a-a2a5c00671cf</v>
       </c>
       <c r="B2" t="str">
-        <v>0368980079</v>
+        <v>0901000011</v>
       </c>
       <c r="C2" t="str">
-        <v>trial</v>
+        <v>weekly</v>
       </c>
       <c r="D2" t="str">
         <v>cutting</v>
@@ -461,30 +461,27 @@
         <v>active</v>
       </c>
       <c r="G2">
-        <v>50000</v>
+        <v>0</v>
       </c>
       <c r="H2">
-        <v>300000</v>
-      </c>
-      <c r="I2">
-        <v>4</v>
+        <v>500000</v>
       </c>
       <c r="J2" t="str">
-        <v>2026-05-09T00:00:00.000Z</v>
+        <v>2026-04-14T00:00:00.000Z</v>
       </c>
       <c r="K2" t="str">
-        <v>2026-05-14T17:00:00.000Z</v>
+        <v>2026-04-20T17:00:00.000Z</v>
       </c>
       <c r="M2" t="str">
-        <v>2026-05-09T04:31:21.529Z</v>
+        <v>2026-05-09T07:05:28.676Z</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>test-sub-0901000001</v>
+        <v>956fd1e2-bec1-4dd9-8f05-fddc317760c9</v>
       </c>
       <c r="B3" t="str">
-        <v>0901000001</v>
+        <v>0901000011</v>
       </c>
       <c r="C3" t="str">
         <v>weekly</v>
@@ -502,68 +499,68 @@
         <v>0</v>
       </c>
       <c r="H3">
-        <v>700000</v>
+        <v>500000</v>
       </c>
       <c r="J3" t="str">
-        <v>2026-04-19T17:00:00.000Z</v>
+        <v>2026-01-05T00:00:00.000Z</v>
       </c>
       <c r="K3" t="str">
-        <v>2026-05-10T17:00:00.000Z</v>
+        <v>2026-01-11T17:00:00.000Z</v>
       </c>
       <c r="M3" t="str">
-        <v>2026-05-09T04:27:53.254Z</v>
+        <v>2026-05-09T07:05:19.463Z</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>test-sub-0901000002</v>
+        <v>11c91237-dccb-42a1-a7a9-145b30159d2e</v>
       </c>
       <c r="B4" t="str">
-        <v>0901000002</v>
+        <v>0901000011</v>
       </c>
       <c r="C4" t="str">
-        <v>monthly</v>
+        <v>weekly</v>
       </c>
       <c r="D4" t="str">
-        <v>maintenance</v>
+        <v>cutting</v>
       </c>
       <c r="E4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F4" t="str">
         <v>active</v>
       </c>
       <c r="G4">
-        <v>30000</v>
+        <v>0</v>
       </c>
       <c r="H4">
-        <v>2600000</v>
+        <v>500000</v>
       </c>
       <c r="J4" t="str">
-        <v>2026-04-19T17:00:00.000Z</v>
+        <v>2026-03-09T00:00:00.000Z</v>
       </c>
       <c r="K4" t="str">
-        <v>2026-05-11T17:00:00.000Z</v>
+        <v>2026-03-15T17:00:00.000Z</v>
       </c>
       <c r="M4" t="str">
-        <v>2026-05-09T04:27:53.255Z</v>
+        <v>2026-05-09T07:05:09.744Z</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>test-sub-0901000003</v>
+        <v>e01d987d-6a5f-4f31-bd71-1486afa53c78</v>
       </c>
       <c r="B5" t="str">
-        <v>0901000003</v>
+        <v>0368980079</v>
       </c>
       <c r="C5" t="str">
-        <v>weekly</v>
+        <v>trial</v>
       </c>
       <c r="D5" t="str">
-        <v>bulking</v>
+        <v>cutting</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F5" t="str">
         <v>active</v>
@@ -572,27 +569,30 @@
         <v>50000</v>
       </c>
       <c r="H5">
-        <v>700000</v>
+        <v>300000</v>
+      </c>
+      <c r="I5">
+        <v>4</v>
       </c>
       <c r="J5" t="str">
-        <v>2026-04-16T17:00:00.000Z</v>
+        <v>2026-05-09T00:00:00.000Z</v>
       </c>
       <c r="K5" t="str">
-        <v>2026-05-13T17:00:00.000Z</v>
+        <v>2026-05-14T17:00:00.000Z</v>
       </c>
       <c r="M5" t="str">
-        <v>2026-05-09T04:27:53.255Z</v>
+        <v>2026-05-09T04:31:21.529Z</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>test-sub-0901000004</v>
+        <v>test-sub-0901000001</v>
       </c>
       <c r="B6" t="str">
-        <v>0901000004</v>
+        <v>0901000001</v>
       </c>
       <c r="C6" t="str">
-        <v>monthly</v>
+        <v>weekly</v>
       </c>
       <c r="D6" t="str">
         <v>cutting</v>
@@ -607,27 +607,27 @@
         <v>0</v>
       </c>
       <c r="H6">
-        <v>2600000</v>
+        <v>700000</v>
       </c>
       <c r="J6" t="str">
-        <v>2026-04-15T17:00:00.000Z</v>
+        <v>2026-04-19T17:00:00.000Z</v>
       </c>
       <c r="K6" t="str">
-        <v>2026-05-17T17:00:00.000Z</v>
+        <v>2026-05-10T17:00:00.000Z</v>
       </c>
       <c r="M6" t="str">
-        <v>2026-05-09T04:27:53.255Z</v>
+        <v>2026-05-09T04:27:53.254Z</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>test-sub-0901000005</v>
+        <v>test-sub-0901000002</v>
       </c>
       <c r="B7" t="str">
-        <v>0901000005</v>
+        <v>0901000002</v>
       </c>
       <c r="C7" t="str">
-        <v>weekly</v>
+        <v>monthly</v>
       </c>
       <c r="D7" t="str">
         <v>maintenance</v>
@@ -642,13 +642,13 @@
         <v>30000</v>
       </c>
       <c r="H7">
-        <v>700000</v>
+        <v>2600000</v>
       </c>
       <c r="J7" t="str">
-        <v>2026-04-14T17:00:00.000Z</v>
+        <v>2026-04-19T17:00:00.000Z</v>
       </c>
       <c r="K7" t="str">
-        <v>2026-05-17T17:00:00.000Z</v>
+        <v>2026-05-11T17:00:00.000Z</v>
       </c>
       <c r="M7" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -656,13 +656,13 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>test-sub-0901000006</v>
+        <v>test-sub-0901000003</v>
       </c>
       <c r="B8" t="str">
-        <v>0901000006</v>
+        <v>0901000003</v>
       </c>
       <c r="C8" t="str">
-        <v>monthly</v>
+        <v>weekly</v>
       </c>
       <c r="D8" t="str">
         <v>bulking</v>
@@ -674,16 +674,16 @@
         <v>active</v>
       </c>
       <c r="G8">
-        <v>0</v>
+        <v>50000</v>
       </c>
       <c r="H8">
-        <v>2600000</v>
+        <v>700000</v>
       </c>
       <c r="J8" t="str">
-        <v>2026-04-13T17:00:00.000Z</v>
+        <v>2026-04-16T17:00:00.000Z</v>
       </c>
       <c r="K8" t="str">
-        <v>2026-05-18T17:00:00.000Z</v>
+        <v>2026-05-13T17:00:00.000Z</v>
       </c>
       <c r="M8" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -691,13 +691,13 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>test-sub-0901000007</v>
+        <v>test-sub-0901000004</v>
       </c>
       <c r="B9" t="str">
-        <v>0901000007</v>
+        <v>0901000004</v>
       </c>
       <c r="C9" t="str">
-        <v>weekly</v>
+        <v>monthly</v>
       </c>
       <c r="D9" t="str">
         <v>cutting</v>
@@ -709,16 +709,16 @@
         <v>active</v>
       </c>
       <c r="G9">
-        <v>30000</v>
+        <v>0</v>
       </c>
       <c r="H9">
-        <v>700000</v>
+        <v>2600000</v>
       </c>
       <c r="J9" t="str">
-        <v>2026-04-12T17:00:00.000Z</v>
+        <v>2026-04-15T17:00:00.000Z</v>
       </c>
       <c r="K9" t="str">
-        <v>2026-05-20T17:00:00.000Z</v>
+        <v>2026-05-17T17:00:00.000Z</v>
       </c>
       <c r="M9" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -726,13 +726,13 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>test-sub-0901000008</v>
+        <v>test-sub-0901000005</v>
       </c>
       <c r="B10" t="str">
-        <v>0901000008</v>
+        <v>0901000005</v>
       </c>
       <c r="C10" t="str">
-        <v>monthly</v>
+        <v>weekly</v>
       </c>
       <c r="D10" t="str">
         <v>maintenance</v>
@@ -744,16 +744,16 @@
         <v>active</v>
       </c>
       <c r="G10">
-        <v>50000</v>
+        <v>30000</v>
       </c>
       <c r="H10">
-        <v>2600000</v>
+        <v>700000</v>
       </c>
       <c r="J10" t="str">
-        <v>2026-04-12T17:00:00.000Z</v>
+        <v>2026-04-14T17:00:00.000Z</v>
       </c>
       <c r="K10" t="str">
-        <v>2026-05-24T17:00:00.000Z</v>
+        <v>2026-05-17T17:00:00.000Z</v>
       </c>
       <c r="M10" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -761,13 +761,13 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>test-sub-0901000009</v>
+        <v>test-sub-0901000006</v>
       </c>
       <c r="B11" t="str">
-        <v>0901000009</v>
+        <v>0901000006</v>
       </c>
       <c r="C11" t="str">
-        <v>weekly</v>
+        <v>monthly</v>
       </c>
       <c r="D11" t="str">
         <v>bulking</v>
@@ -782,13 +782,13 @@
         <v>0</v>
       </c>
       <c r="H11">
-        <v>700000</v>
+        <v>2600000</v>
       </c>
       <c r="J11" t="str">
-        <v>2026-04-12T17:00:00.000Z</v>
+        <v>2026-04-13T17:00:00.000Z</v>
       </c>
       <c r="K11" t="str">
-        <v>2026-05-24T17:00:00.000Z</v>
+        <v>2026-05-18T17:00:00.000Z</v>
       </c>
       <c r="M11" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -796,13 +796,13 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>test-sub-0901000010</v>
+        <v>test-sub-0901000007</v>
       </c>
       <c r="B12" t="str">
-        <v>0901000010</v>
+        <v>0901000007</v>
       </c>
       <c r="C12" t="str">
-        <v>monthly</v>
+        <v>weekly</v>
       </c>
       <c r="D12" t="str">
         <v>cutting</v>
@@ -817,13 +817,13 @@
         <v>30000</v>
       </c>
       <c r="H12">
-        <v>2600000</v>
+        <v>700000</v>
       </c>
       <c r="J12" t="str">
-        <v>2026-04-09T17:00:00.000Z</v>
+        <v>2026-04-12T17:00:00.000Z</v>
       </c>
       <c r="K12" t="str">
-        <v>2026-05-24T17:00:00.000Z</v>
+        <v>2026-05-20T17:00:00.000Z</v>
       </c>
       <c r="M12" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -831,13 +831,13 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>test-sub-0901000011</v>
+        <v>test-sub-0901000008</v>
       </c>
       <c r="B13" t="str">
-        <v>0901000011</v>
+        <v>0901000008</v>
       </c>
       <c r="C13" t="str">
-        <v>weekly</v>
+        <v>monthly</v>
       </c>
       <c r="D13" t="str">
         <v>maintenance</v>
@@ -849,16 +849,16 @@
         <v>active</v>
       </c>
       <c r="G13">
-        <v>0</v>
+        <v>50000</v>
       </c>
       <c r="H13">
-        <v>700000</v>
+        <v>2600000</v>
       </c>
       <c r="J13" t="str">
-        <v>2026-04-19T17:00:00.000Z</v>
+        <v>2026-04-12T17:00:00.000Z</v>
       </c>
       <c r="K13" t="str">
-        <v>2026-05-26T17:00:00.000Z</v>
+        <v>2026-05-24T17:00:00.000Z</v>
       </c>
       <c r="M13" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -866,13 +866,13 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>test-sub-0901000012</v>
+        <v>test-sub-0901000009</v>
       </c>
       <c r="B14" t="str">
-        <v>0901000012</v>
+        <v>0901000009</v>
       </c>
       <c r="C14" t="str">
-        <v>monthly</v>
+        <v>weekly</v>
       </c>
       <c r="D14" t="str">
         <v>bulking</v>
@@ -884,16 +884,16 @@
         <v>active</v>
       </c>
       <c r="G14">
-        <v>30000</v>
+        <v>0</v>
       </c>
       <c r="H14">
-        <v>2600000</v>
+        <v>700000</v>
       </c>
       <c r="J14" t="str">
-        <v>2026-04-19T17:00:00.000Z</v>
+        <v>2026-04-12T17:00:00.000Z</v>
       </c>
       <c r="K14" t="str">
-        <v>2026-05-28T17:00:00.000Z</v>
+        <v>2026-05-24T17:00:00.000Z</v>
       </c>
       <c r="M14" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -901,13 +901,13 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>test-sub-0901000013</v>
+        <v>test-sub-0901000010</v>
       </c>
       <c r="B15" t="str">
-        <v>0901000013</v>
+        <v>0901000010</v>
       </c>
       <c r="C15" t="str">
-        <v>weekly</v>
+        <v>monthly</v>
       </c>
       <c r="D15" t="str">
         <v>cutting</v>
@@ -919,16 +919,16 @@
         <v>active</v>
       </c>
       <c r="G15">
-        <v>50000</v>
+        <v>30000</v>
       </c>
       <c r="H15">
-        <v>700000</v>
+        <v>2600000</v>
       </c>
       <c r="J15" t="str">
-        <v>2026-04-16T17:00:00.000Z</v>
+        <v>2026-04-09T17:00:00.000Z</v>
       </c>
       <c r="K15" t="str">
-        <v>2026-05-31T17:00:00.000Z</v>
+        <v>2026-05-24T17:00:00.000Z</v>
       </c>
       <c r="M15" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -936,19 +936,19 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>test-sub-0901000014</v>
+        <v>test-sub-0901000011</v>
       </c>
       <c r="B16" t="str">
-        <v>0901000014</v>
+        <v>0901000011</v>
       </c>
       <c r="C16" t="str">
-        <v>monthly</v>
+        <v>weekly</v>
       </c>
       <c r="D16" t="str">
         <v>maintenance</v>
       </c>
       <c r="E16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F16" t="str">
         <v>active</v>
@@ -957,13 +957,13 @@
         <v>0</v>
       </c>
       <c r="H16">
-        <v>2600000</v>
+        <v>700000</v>
       </c>
       <c r="J16" t="str">
-        <v>2026-04-15T17:00:00.000Z</v>
+        <v>2026-04-19T00:00:00.000Z</v>
       </c>
       <c r="K16" t="str">
-        <v>2026-05-31T17:00:00.000Z</v>
+        <v>2026-05-26T00:00:00.000Z</v>
       </c>
       <c r="M16" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -971,13 +971,13 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>test-sub-0901000015</v>
+        <v>test-sub-0901000012</v>
       </c>
       <c r="B17" t="str">
-        <v>0901000015</v>
+        <v>0901000012</v>
       </c>
       <c r="C17" t="str">
-        <v>weekly</v>
+        <v>monthly</v>
       </c>
       <c r="D17" t="str">
         <v>bulking</v>
@@ -992,13 +992,13 @@
         <v>30000</v>
       </c>
       <c r="H17">
-        <v>700000</v>
+        <v>2600000</v>
       </c>
       <c r="J17" t="str">
-        <v>2026-04-14T17:00:00.000Z</v>
+        <v>2026-04-19T17:00:00.000Z</v>
       </c>
       <c r="K17" t="str">
-        <v>2026-06-01T17:00:00.000Z</v>
+        <v>2026-05-28T17:00:00.000Z</v>
       </c>
       <c r="M17" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -1006,13 +1006,13 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>test-sub-0901000016</v>
+        <v>test-sub-0901000013</v>
       </c>
       <c r="B18" t="str">
-        <v>0901000016</v>
+        <v>0901000013</v>
       </c>
       <c r="C18" t="str">
-        <v>monthly</v>
+        <v>weekly</v>
       </c>
       <c r="D18" t="str">
         <v>cutting</v>
@@ -1024,16 +1024,16 @@
         <v>active</v>
       </c>
       <c r="G18">
-        <v>0</v>
+        <v>50000</v>
       </c>
       <c r="H18">
-        <v>2600000</v>
+        <v>700000</v>
       </c>
       <c r="J18" t="str">
-        <v>2026-04-13T17:00:00.000Z</v>
+        <v>2026-04-16T17:00:00.000Z</v>
       </c>
       <c r="K18" t="str">
-        <v>2026-06-02T17:00:00.000Z</v>
+        <v>2026-05-31T17:00:00.000Z</v>
       </c>
       <c r="M18" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -1041,13 +1041,13 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>test-sub-0901000017</v>
+        <v>test-sub-0901000014</v>
       </c>
       <c r="B19" t="str">
-        <v>0901000017</v>
+        <v>0901000014</v>
       </c>
       <c r="C19" t="str">
-        <v>weekly</v>
+        <v>monthly</v>
       </c>
       <c r="D19" t="str">
         <v>maintenance</v>
@@ -1059,16 +1059,16 @@
         <v>active</v>
       </c>
       <c r="G19">
-        <v>30000</v>
+        <v>0</v>
       </c>
       <c r="H19">
-        <v>700000</v>
+        <v>2600000</v>
       </c>
       <c r="J19" t="str">
-        <v>2026-04-12T17:00:00.000Z</v>
+        <v>2026-04-15T17:00:00.000Z</v>
       </c>
       <c r="K19" t="str">
-        <v>2026-06-03T17:00:00.000Z</v>
+        <v>2026-05-31T17:00:00.000Z</v>
       </c>
       <c r="M19" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -1076,13 +1076,13 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>test-sub-0901000018</v>
+        <v>test-sub-0901000015</v>
       </c>
       <c r="B20" t="str">
-        <v>0901000018</v>
+        <v>0901000015</v>
       </c>
       <c r="C20" t="str">
-        <v>monthly</v>
+        <v>weekly</v>
       </c>
       <c r="D20" t="str">
         <v>bulking</v>
@@ -1094,16 +1094,16 @@
         <v>active</v>
       </c>
       <c r="G20">
-        <v>50000</v>
+        <v>30000</v>
       </c>
       <c r="H20">
-        <v>2600000</v>
+        <v>700000</v>
       </c>
       <c r="J20" t="str">
-        <v>2026-04-12T17:00:00.000Z</v>
+        <v>2026-04-14T17:00:00.000Z</v>
       </c>
       <c r="K20" t="str">
-        <v>2026-06-07T17:00:00.000Z</v>
+        <v>2026-06-01T17:00:00.000Z</v>
       </c>
       <c r="M20" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -1111,13 +1111,13 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>test-sub-0901000019</v>
+        <v>test-sub-0901000016</v>
       </c>
       <c r="B21" t="str">
-        <v>0901000019</v>
+        <v>0901000016</v>
       </c>
       <c r="C21" t="str">
-        <v>weekly</v>
+        <v>monthly</v>
       </c>
       <c r="D21" t="str">
         <v>cutting</v>
@@ -1132,13 +1132,13 @@
         <v>0</v>
       </c>
       <c r="H21">
-        <v>700000</v>
+        <v>2600000</v>
       </c>
       <c r="J21" t="str">
-        <v>2026-04-12T17:00:00.000Z</v>
+        <v>2026-04-13T17:00:00.000Z</v>
       </c>
       <c r="K21" t="str">
-        <v>2026-06-07T17:00:00.000Z</v>
+        <v>2026-06-02T17:00:00.000Z</v>
       </c>
       <c r="M21" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -1146,13 +1146,13 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>test-sub-0901000020</v>
+        <v>test-sub-0901000017</v>
       </c>
       <c r="B22" t="str">
-        <v>0901000020</v>
+        <v>0901000017</v>
       </c>
       <c r="C22" t="str">
-        <v>monthly</v>
+        <v>weekly</v>
       </c>
       <c r="D22" t="str">
         <v>maintenance</v>
@@ -1167,13 +1167,13 @@
         <v>30000</v>
       </c>
       <c r="H22">
-        <v>2600000</v>
+        <v>700000</v>
       </c>
       <c r="J22" t="str">
-        <v>2026-04-09T17:00:00.000Z</v>
+        <v>2026-04-12T17:00:00.000Z</v>
       </c>
       <c r="K22" t="str">
-        <v>2026-06-09T17:00:00.000Z</v>
+        <v>2026-06-03T17:00:00.000Z</v>
       </c>
       <c r="M22" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -1181,13 +1181,13 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>test-sub-0901000021</v>
+        <v>test-sub-0901000018</v>
       </c>
       <c r="B23" t="str">
-        <v>0901000021</v>
+        <v>0901000018</v>
       </c>
       <c r="C23" t="str">
-        <v>weekly</v>
+        <v>monthly</v>
       </c>
       <c r="D23" t="str">
         <v>bulking</v>
@@ -1199,16 +1199,16 @@
         <v>active</v>
       </c>
       <c r="G23">
-        <v>0</v>
+        <v>50000</v>
       </c>
       <c r="H23">
-        <v>700000</v>
+        <v>2600000</v>
       </c>
       <c r="J23" t="str">
-        <v>2026-04-19T17:00:00.000Z</v>
+        <v>2026-04-12T17:00:00.000Z</v>
       </c>
       <c r="K23" t="str">
-        <v>2026-06-14T17:00:00.000Z</v>
+        <v>2026-06-07T17:00:00.000Z</v>
       </c>
       <c r="M23" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -1216,13 +1216,13 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>test-sub-0901000022</v>
+        <v>test-sub-0901000019</v>
       </c>
       <c r="B24" t="str">
-        <v>0901000022</v>
+        <v>0901000019</v>
       </c>
       <c r="C24" t="str">
-        <v>monthly</v>
+        <v>weekly</v>
       </c>
       <c r="D24" t="str">
         <v>cutting</v>
@@ -1234,16 +1234,16 @@
         <v>active</v>
       </c>
       <c r="G24">
-        <v>30000</v>
+        <v>0</v>
       </c>
       <c r="H24">
-        <v>2600000</v>
+        <v>700000</v>
       </c>
       <c r="J24" t="str">
-        <v>2026-04-19T17:00:00.000Z</v>
+        <v>2026-04-12T17:00:00.000Z</v>
       </c>
       <c r="K24" t="str">
-        <v>2026-06-15T17:00:00.000Z</v>
+        <v>2026-06-07T17:00:00.000Z</v>
       </c>
       <c r="M24" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -1251,13 +1251,13 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>test-sub-0901000023</v>
+        <v>test-sub-0901000020</v>
       </c>
       <c r="B25" t="str">
-        <v>0901000023</v>
+        <v>0901000020</v>
       </c>
       <c r="C25" t="str">
-        <v>weekly</v>
+        <v>monthly</v>
       </c>
       <c r="D25" t="str">
         <v>maintenance</v>
@@ -1269,16 +1269,16 @@
         <v>active</v>
       </c>
       <c r="G25">
-        <v>50000</v>
+        <v>30000</v>
       </c>
       <c r="H25">
-        <v>700000</v>
+        <v>2600000</v>
       </c>
       <c r="J25" t="str">
-        <v>2026-04-16T17:00:00.000Z</v>
+        <v>2026-04-09T17:00:00.000Z</v>
       </c>
       <c r="K25" t="str">
-        <v>2026-06-17T17:00:00.000Z</v>
+        <v>2026-06-09T17:00:00.000Z</v>
       </c>
       <c r="M25" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -1286,13 +1286,13 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>test-sub-0901000024</v>
+        <v>test-sub-0901000021</v>
       </c>
       <c r="B26" t="str">
-        <v>0901000024</v>
+        <v>0901000021</v>
       </c>
       <c r="C26" t="str">
-        <v>monthly</v>
+        <v>weekly</v>
       </c>
       <c r="D26" t="str">
         <v>bulking</v>
@@ -1307,13 +1307,13 @@
         <v>0</v>
       </c>
       <c r="H26">
-        <v>2600000</v>
+        <v>700000</v>
       </c>
       <c r="J26" t="str">
-        <v>2026-04-15T17:00:00.000Z</v>
+        <v>2026-04-19T17:00:00.000Z</v>
       </c>
       <c r="K26" t="str">
-        <v>2026-06-21T17:00:00.000Z</v>
+        <v>2026-06-14T17:00:00.000Z</v>
       </c>
       <c r="M26" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -1321,13 +1321,13 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>test-sub-0901000025</v>
+        <v>test-sub-0901000022</v>
       </c>
       <c r="B27" t="str">
-        <v>0901000025</v>
+        <v>0901000022</v>
       </c>
       <c r="C27" t="str">
-        <v>weekly</v>
+        <v>monthly</v>
       </c>
       <c r="D27" t="str">
         <v>cutting</v>
@@ -1342,13 +1342,13 @@
         <v>30000</v>
       </c>
       <c r="H27">
-        <v>700000</v>
+        <v>2600000</v>
       </c>
       <c r="J27" t="str">
-        <v>2026-04-14T17:00:00.000Z</v>
+        <v>2026-04-19T17:00:00.000Z</v>
       </c>
       <c r="K27" t="str">
-        <v>2026-06-22T17:00:00.000Z</v>
+        <v>2026-06-15T17:00:00.000Z</v>
       </c>
       <c r="M27" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -1356,13 +1356,13 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>test-sub-0901000026</v>
+        <v>test-sub-0901000023</v>
       </c>
       <c r="B28" t="str">
-        <v>0901000026</v>
+        <v>0901000023</v>
       </c>
       <c r="C28" t="str">
-        <v>monthly</v>
+        <v>weekly</v>
       </c>
       <c r="D28" t="str">
         <v>maintenance</v>
@@ -1374,16 +1374,16 @@
         <v>active</v>
       </c>
       <c r="G28">
-        <v>0</v>
+        <v>50000</v>
       </c>
       <c r="H28">
-        <v>2600000</v>
+        <v>700000</v>
       </c>
       <c r="J28" t="str">
-        <v>2026-04-13T17:00:00.000Z</v>
+        <v>2026-04-16T17:00:00.000Z</v>
       </c>
       <c r="K28" t="str">
-        <v>2026-05-13T17:00:00.000Z</v>
+        <v>2026-06-17T17:00:00.000Z</v>
       </c>
       <c r="M28" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -1391,13 +1391,13 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>test-sub-0901000027</v>
+        <v>test-sub-0901000024</v>
       </c>
       <c r="B29" t="str">
-        <v>0901000027</v>
+        <v>0901000024</v>
       </c>
       <c r="C29" t="str">
-        <v>weekly</v>
+        <v>monthly</v>
       </c>
       <c r="D29" t="str">
         <v>bulking</v>
@@ -1409,16 +1409,16 @@
         <v>active</v>
       </c>
       <c r="G29">
-        <v>30000</v>
+        <v>0</v>
       </c>
       <c r="H29">
-        <v>700000</v>
+        <v>2600000</v>
       </c>
       <c r="J29" t="str">
-        <v>2026-04-12T17:00:00.000Z</v>
+        <v>2026-04-15T17:00:00.000Z</v>
       </c>
       <c r="K29" t="str">
-        <v>2026-05-17T17:00:00.000Z</v>
+        <v>2026-06-21T17:00:00.000Z</v>
       </c>
       <c r="M29" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -1426,13 +1426,13 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>test-sub-0901000028</v>
+        <v>test-sub-0901000025</v>
       </c>
       <c r="B30" t="str">
-        <v>0901000028</v>
+        <v>0901000025</v>
       </c>
       <c r="C30" t="str">
-        <v>monthly</v>
+        <v>weekly</v>
       </c>
       <c r="D30" t="str">
         <v>cutting</v>
@@ -1444,16 +1444,16 @@
         <v>active</v>
       </c>
       <c r="G30">
-        <v>50000</v>
+        <v>30000</v>
       </c>
       <c r="H30">
-        <v>2600000</v>
+        <v>700000</v>
       </c>
       <c r="J30" t="str">
-        <v>2026-04-12T17:00:00.000Z</v>
+        <v>2026-04-14T17:00:00.000Z</v>
       </c>
       <c r="K30" t="str">
-        <v>2026-05-18T17:00:00.000Z</v>
+        <v>2026-06-22T17:00:00.000Z</v>
       </c>
       <c r="M30" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -1461,13 +1461,13 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>test-sub-0901000029</v>
+        <v>test-sub-0901000026</v>
       </c>
       <c r="B31" t="str">
-        <v>0901000029</v>
+        <v>0901000026</v>
       </c>
       <c r="C31" t="str">
-        <v>weekly</v>
+        <v>monthly</v>
       </c>
       <c r="D31" t="str">
         <v>maintenance</v>
@@ -1482,13 +1482,13 @@
         <v>0</v>
       </c>
       <c r="H31">
-        <v>700000</v>
+        <v>2600000</v>
       </c>
       <c r="J31" t="str">
-        <v>2026-04-12T17:00:00.000Z</v>
+        <v>2026-04-13T17:00:00.000Z</v>
       </c>
       <c r="K31" t="str">
-        <v>2026-05-24T17:00:00.000Z</v>
+        <v>2026-05-13T17:00:00.000Z</v>
       </c>
       <c r="M31" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -1496,13 +1496,13 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>test-sub-0901000030</v>
+        <v>test-sub-0901000027</v>
       </c>
       <c r="B32" t="str">
-        <v>0901000030</v>
+        <v>0901000027</v>
       </c>
       <c r="C32" t="str">
-        <v>monthly</v>
+        <v>weekly</v>
       </c>
       <c r="D32" t="str">
         <v>bulking</v>
@@ -1517,13 +1517,13 @@
         <v>30000</v>
       </c>
       <c r="H32">
-        <v>2600000</v>
+        <v>700000</v>
       </c>
       <c r="J32" t="str">
-        <v>2026-04-09T17:00:00.000Z</v>
+        <v>2026-04-12T17:00:00.000Z</v>
       </c>
       <c r="K32" t="str">
-        <v>2026-05-28T17:00:00.000Z</v>
+        <v>2026-05-17T17:00:00.000Z</v>
       </c>
       <c r="M32" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -1531,37 +1531,34 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>test-sub-0901000031</v>
+        <v>test-sub-0901000028</v>
       </c>
       <c r="B33" t="str">
-        <v>0901000031</v>
+        <v>0901000028</v>
       </c>
       <c r="C33" t="str">
         <v>monthly</v>
       </c>
       <c r="D33" t="str">
-        <v>maintenance</v>
+        <v>cutting</v>
       </c>
       <c r="E33">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F33" t="str">
-        <v>cancelled</v>
+        <v>active</v>
       </c>
       <c r="G33">
         <v>50000</v>
       </c>
       <c r="H33">
-        <v>1000000</v>
+        <v>2600000</v>
       </c>
       <c r="J33" t="str">
-        <v>2026-04-19T17:00:00.000Z</v>
+        <v>2026-04-12T17:00:00.000Z</v>
       </c>
       <c r="K33" t="str">
-        <v>2026-05-05T17:00:00.000Z</v>
-      </c>
-      <c r="L33" t="str">
-        <v>Đi du lịch dài ngày</v>
+        <v>2026-05-18T17:00:00.000Z</v>
       </c>
       <c r="M33" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -1569,13 +1566,13 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>test-sub-0901000032</v>
+        <v>test-sub-0901000029</v>
       </c>
       <c r="B34" t="str">
-        <v>0901000032</v>
+        <v>0901000029</v>
       </c>
       <c r="C34" t="str">
-        <v>monthly</v>
+        <v>weekly</v>
       </c>
       <c r="D34" t="str">
         <v>maintenance</v>
@@ -1584,22 +1581,19 @@
         <v>1</v>
       </c>
       <c r="F34" t="str">
-        <v>cancelled</v>
+        <v>active</v>
       </c>
       <c r="G34">
-        <v>50000</v>
+        <v>0</v>
       </c>
       <c r="H34">
-        <v>1000000</v>
+        <v>700000</v>
       </c>
       <c r="J34" t="str">
-        <v>2026-04-19T17:00:00.000Z</v>
+        <v>2026-04-12T17:00:00.000Z</v>
       </c>
       <c r="K34" t="str">
-        <v>2026-04-28T17:00:00.000Z</v>
-      </c>
-      <c r="L34" t="str">
-        <v>Tài chính</v>
+        <v>2026-05-24T17:00:00.000Z</v>
       </c>
       <c r="M34" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -1607,37 +1601,34 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>test-sub-0901000033</v>
+        <v>test-sub-0901000030</v>
       </c>
       <c r="B35" t="str">
-        <v>0901000033</v>
+        <v>0901000030</v>
       </c>
       <c r="C35" t="str">
         <v>monthly</v>
       </c>
       <c r="D35" t="str">
-        <v>maintenance</v>
+        <v>bulking</v>
       </c>
       <c r="E35">
         <v>1</v>
       </c>
       <c r="F35" t="str">
-        <v>cancelled</v>
+        <v>active</v>
       </c>
       <c r="G35">
-        <v>50000</v>
+        <v>30000</v>
       </c>
       <c r="H35">
-        <v>1000000</v>
+        <v>2600000</v>
       </c>
       <c r="J35" t="str">
-        <v>2026-04-19T17:00:00.000Z</v>
+        <v>2026-04-09T17:00:00.000Z</v>
       </c>
       <c r="K35" t="str">
-        <v>2026-05-03T17:00:00.000Z</v>
-      </c>
-      <c r="L35" t="str">
-        <v>Không hài lòng</v>
+        <v>2026-05-28T17:00:00.000Z</v>
       </c>
       <c r="M35" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -1645,10 +1636,10 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>test-sub-0901000034</v>
+        <v>test-sub-0901000031</v>
       </c>
       <c r="B36" t="str">
-        <v>0901000034</v>
+        <v>0901000031</v>
       </c>
       <c r="C36" t="str">
         <v>monthly</v>
@@ -1672,10 +1663,10 @@
         <v>2026-04-19T17:00:00.000Z</v>
       </c>
       <c r="K36" t="str">
-        <v>2026-04-19T17:00:00.000Z</v>
+        <v>2026-05-05T17:00:00.000Z</v>
       </c>
       <c r="L36" t="str">
-        <v>Chuyển nhà xa</v>
+        <v>Đi du lịch dài ngày</v>
       </c>
       <c r="M36" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -1683,10 +1674,10 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>test-sub-0901000035</v>
+        <v>test-sub-0901000032</v>
       </c>
       <c r="B37" t="str">
-        <v>0901000035</v>
+        <v>0901000032</v>
       </c>
       <c r="C37" t="str">
         <v>monthly</v>
@@ -1710,10 +1701,10 @@
         <v>2026-04-19T17:00:00.000Z</v>
       </c>
       <c r="K37" t="str">
-        <v>2026-05-07T17:00:00.000Z</v>
+        <v>2026-04-28T17:00:00.000Z</v>
       </c>
       <c r="L37" t="str">
-        <v>Hết nhu cầu</v>
+        <v>Tài chính</v>
       </c>
       <c r="M37" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -1721,10 +1712,10 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>test-sub-0901000036</v>
+        <v>test-sub-0901000033</v>
       </c>
       <c r="B38" t="str">
-        <v>0901000036</v>
+        <v>0901000033</v>
       </c>
       <c r="C38" t="str">
         <v>monthly</v>
@@ -1748,10 +1739,10 @@
         <v>2026-04-19T17:00:00.000Z</v>
       </c>
       <c r="K38" t="str">
-        <v>2026-04-30T17:00:00.000Z</v>
+        <v>2026-05-03T17:00:00.000Z</v>
       </c>
       <c r="L38" t="str">
-        <v>Mang thai</v>
+        <v>Không hài lòng</v>
       </c>
       <c r="M38" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -1759,10 +1750,10 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>test-sub-0901000037</v>
+        <v>test-sub-0901000034</v>
       </c>
       <c r="B39" t="str">
-        <v>0901000037</v>
+        <v>0901000034</v>
       </c>
       <c r="C39" t="str">
         <v>monthly</v>
@@ -1786,10 +1777,10 @@
         <v>2026-04-19T17:00:00.000Z</v>
       </c>
       <c r="K39" t="str">
-        <v>2026-04-23T17:00:00.000Z</v>
+        <v>2026-04-19T17:00:00.000Z</v>
       </c>
       <c r="L39" t="str">
-        <v>Đổi chế độ ăn</v>
+        <v>Chuyển nhà xa</v>
       </c>
       <c r="M39" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -1797,10 +1788,10 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>test-sub-0901000038</v>
+        <v>test-sub-0901000035</v>
       </c>
       <c r="B40" t="str">
-        <v>0901000038</v>
+        <v>0901000035</v>
       </c>
       <c r="C40" t="str">
         <v>monthly</v>
@@ -1824,10 +1815,10 @@
         <v>2026-04-19T17:00:00.000Z</v>
       </c>
       <c r="K40" t="str">
-        <v>2026-05-03T17:00:00.000Z</v>
+        <v>2026-05-07T17:00:00.000Z</v>
       </c>
       <c r="L40" t="str">
-        <v>Công việc bận rộn</v>
+        <v>Hết nhu cầu</v>
       </c>
       <c r="M40" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -1835,10 +1826,10 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>test-sub-0901000039</v>
+        <v>test-sub-0901000036</v>
       </c>
       <c r="B41" t="str">
-        <v>0901000039</v>
+        <v>0901000036</v>
       </c>
       <c r="C41" t="str">
         <v>monthly</v>
@@ -1850,7 +1841,7 @@
         <v>1</v>
       </c>
       <c r="F41" t="str">
-        <v>paused</v>
+        <v>cancelled</v>
       </c>
       <c r="G41">
         <v>50000</v>
@@ -1862,7 +1853,10 @@
         <v>2026-04-19T17:00:00.000Z</v>
       </c>
       <c r="K41" t="str">
-        <v>2026-05-18T17:00:00.000Z</v>
+        <v>2026-04-30T17:00:00.000Z</v>
+      </c>
+      <c r="L41" t="str">
+        <v>Mang thai</v>
       </c>
       <c r="M41" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -1870,10 +1864,10 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>test-sub-0901000040</v>
+        <v>test-sub-0901000037</v>
       </c>
       <c r="B42" t="str">
-        <v>0901000040</v>
+        <v>0901000037</v>
       </c>
       <c r="C42" t="str">
         <v>monthly</v>
@@ -1885,7 +1879,7 @@
         <v>1</v>
       </c>
       <c r="F42" t="str">
-        <v>paused</v>
+        <v>cancelled</v>
       </c>
       <c r="G42">
         <v>50000</v>
@@ -1897,7 +1891,10 @@
         <v>2026-04-19T17:00:00.000Z</v>
       </c>
       <c r="K42" t="str">
-        <v>2026-05-24T17:00:00.000Z</v>
+        <v>2026-04-23T17:00:00.000Z</v>
+      </c>
+      <c r="L42" t="str">
+        <v>Đổi chế độ ăn</v>
       </c>
       <c r="M42" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -1905,10 +1902,10 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>test-sub-0901000041</v>
+        <v>test-sub-0901000038</v>
       </c>
       <c r="B43" t="str">
-        <v>0901000041</v>
+        <v>0901000038</v>
       </c>
       <c r="C43" t="str">
         <v>monthly</v>
@@ -1920,7 +1917,7 @@
         <v>1</v>
       </c>
       <c r="F43" t="str">
-        <v>paused</v>
+        <v>cancelled</v>
       </c>
       <c r="G43">
         <v>50000</v>
@@ -1932,7 +1929,10 @@
         <v>2026-04-19T17:00:00.000Z</v>
       </c>
       <c r="K43" t="str">
-        <v>2026-05-28T17:00:00.000Z</v>
+        <v>2026-05-03T17:00:00.000Z</v>
+      </c>
+      <c r="L43" t="str">
+        <v>Công việc bận rộn</v>
       </c>
       <c r="M43" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -1940,10 +1940,10 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>test-sub-0901000042</v>
+        <v>test-sub-0901000039</v>
       </c>
       <c r="B44" t="str">
-        <v>0901000042</v>
+        <v>0901000039</v>
       </c>
       <c r="C44" t="str">
         <v>monthly</v>
@@ -1967,7 +1967,7 @@
         <v>2026-04-19T17:00:00.000Z</v>
       </c>
       <c r="K44" t="str">
-        <v>2026-05-17T17:00:00.000Z</v>
+        <v>2026-05-18T17:00:00.000Z</v>
       </c>
       <c r="M44" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -1975,10 +1975,10 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>test-sub-0901000043</v>
+        <v>test-sub-0901000040</v>
       </c>
       <c r="B45" t="str">
-        <v>0901000043</v>
+        <v>0901000040</v>
       </c>
       <c r="C45" t="str">
         <v>monthly</v>
@@ -2002,7 +2002,7 @@
         <v>2026-04-19T17:00:00.000Z</v>
       </c>
       <c r="K45" t="str">
-        <v>2026-05-13T17:00:00.000Z</v>
+        <v>2026-05-24T17:00:00.000Z</v>
       </c>
       <c r="M45" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
@@ -2010,10 +2010,10 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>test-sub-0901000044</v>
+        <v>test-sub-0901000041</v>
       </c>
       <c r="B46" t="str">
-        <v>0901000044</v>
+        <v>0901000041</v>
       </c>
       <c r="C46" t="str">
         <v>monthly</v>
@@ -2037,15 +2037,120 @@
         <v>2026-04-19T17:00:00.000Z</v>
       </c>
       <c r="K46" t="str">
+        <v>2026-05-28T17:00:00.000Z</v>
+      </c>
+      <c r="M46" t="str">
+        <v>2026-05-09T04:27:53.255Z</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>test-sub-0901000042</v>
+      </c>
+      <c r="B47" t="str">
+        <v>0901000042</v>
+      </c>
+      <c r="C47" t="str">
+        <v>monthly</v>
+      </c>
+      <c r="D47" t="str">
+        <v>maintenance</v>
+      </c>
+      <c r="E47">
+        <v>1</v>
+      </c>
+      <c r="F47" t="str">
+        <v>paused</v>
+      </c>
+      <c r="G47">
+        <v>50000</v>
+      </c>
+      <c r="H47">
+        <v>1000000</v>
+      </c>
+      <c r="J47" t="str">
+        <v>2026-04-19T17:00:00.000Z</v>
+      </c>
+      <c r="K47" t="str">
+        <v>2026-05-17T17:00:00.000Z</v>
+      </c>
+      <c r="M47" t="str">
+        <v>2026-05-09T04:27:53.255Z</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>test-sub-0901000043</v>
+      </c>
+      <c r="B48" t="str">
+        <v>0901000043</v>
+      </c>
+      <c r="C48" t="str">
+        <v>monthly</v>
+      </c>
+      <c r="D48" t="str">
+        <v>maintenance</v>
+      </c>
+      <c r="E48">
+        <v>1</v>
+      </c>
+      <c r="F48" t="str">
+        <v>paused</v>
+      </c>
+      <c r="G48">
+        <v>50000</v>
+      </c>
+      <c r="H48">
+        <v>1000000</v>
+      </c>
+      <c r="J48" t="str">
+        <v>2026-04-19T17:00:00.000Z</v>
+      </c>
+      <c r="K48" t="str">
+        <v>2026-05-13T17:00:00.000Z</v>
+      </c>
+      <c r="M48" t="str">
+        <v>2026-05-09T04:27:53.255Z</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>test-sub-0901000044</v>
+      </c>
+      <c r="B49" t="str">
+        <v>0901000044</v>
+      </c>
+      <c r="C49" t="str">
+        <v>monthly</v>
+      </c>
+      <c r="D49" t="str">
+        <v>maintenance</v>
+      </c>
+      <c r="E49">
+        <v>1</v>
+      </c>
+      <c r="F49" t="str">
+        <v>paused</v>
+      </c>
+      <c r="G49">
+        <v>50000</v>
+      </c>
+      <c r="H49">
+        <v>1000000</v>
+      </c>
+      <c r="J49" t="str">
+        <v>2026-04-19T17:00:00.000Z</v>
+      </c>
+      <c r="K49" t="str">
         <v>2026-06-07T17:00:00.000Z</v>
       </c>
-      <c r="M46" t="str">
+      <c r="M49" t="str">
         <v>2026-05-09T04:27:53.255Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M46"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M49"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>